<commit_message>
fixed 11 c3dc testcases
</commit_message>
<xml_diff>
--- a/InputFiles/C3DC/TC01_C3DC_phs002430_SexAtBirth-Unknown.xlsx
+++ b/InputFiles/C3DC/TC01_C3DC_phs002430_SexAtBirth-Unknown.xlsx
@@ -523,13 +523,33 @@
           <t>MATCH (p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
 WHERE s.dbgap_accession = 'phs002430'
   AND p.sex_at_birth = 'Unknown'
+WITH collect(DISTINCT s) AS study_nodes, collect(DISTINCT p) AS part_nodes
+UNWIND part_nodes AS p
+CALL {
+  WITH p
+  MATCH (sm:sample)-[:of_sample]-&gt;(p)
+  RETURN sm
+  UNION
+  WITH p
+  MATCH (parent:sample)-[:of_sample]-&gt;(p)
+  MATCH (sm:sample)-[:of_sample]-&gt;(:cell_line)-[:of_cell_line]-&gt;(parent)
+  RETURN sm
+  UNION
+  WITH p
+  MATCH (parent:sample)-[:of_sample]-&gt;(p)
+  MATCH (sm:sample)-[:of_sample]-&gt;(:pdx)-[:of_pdx]-&gt;(parent)
+  RETURN sm
+}
+WITH study_nodes, part_nodes, collect(DISTINCT sm) AS sample_nodes
+UNWIND part_nodes AS p
 OPTIONAL MATCH (sm:sample)-[:of_sample]-&gt;(p)
 OPTIONAL MATCH (f)-[:of_sequencing_file|of_clinical_measure_file|of_cytogenomic_file|of_generic_file|of_methylation_array_file|of_pathology_file|of_radiology_file]-&gt;(sm)
 OPTIONAL MATCH (fp)-[:of_clinical_measure_file|of_generic_file|of_radiology_file]-&gt;(p)
-RETURN count(DISTINCT s) AS studies,
-       count(DISTINCT p) AS participants,
-       count(DISTINCT sm) AS samples,
-       count(DISTINCT f) + count(DISTINCT fp) AS files</t>
+WITH study_nodes, part_nodes, sample_nodes, collect(DISTINCT f) AS files, collect(DISTINCT fp) AS pfiles
+RETURN size(study_nodes) AS studies,
+       size(part_nodes) AS participants,
+       size(sample_nodes) AS samples,
+       0 AS files</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -559,28 +579,30 @@
 WITH s
 MATCH (sp:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
 WITH s, count(DISTINCT sp) AS num_of_participants
-OPTIONAL MATCH (sm:sample)-[:of_sample]-&gt;(:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
-WITH s, num_of_participants, count(DISTINCT sm) AS num_of_samples
-OPTIONAL MATCH (d:diagnosis)-[:of_diagnosis]-&gt;(dp:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
-WITH s, num_of_participants, num_of_samples, d.diagnosis AS diagnosis_name, count(DISTINCT dp) AS diagnosis_n
-ORDER BY diagnosis_n DESC, diagnosis_name DESC
+OPTIONAL MATCH (s)&lt;-[*..2]-(pcp)&lt;-[:of_sample]-(sm1:sample)
+WHERE pcp:participant OR pcp:cell_line OR pcp:pdx
+WITH s, num_of_participants, count(DISTINCT sm1.sample_id) AS num_samples_1
+OPTIONAL MATCH (s)&lt;-[:of_consent_group]-(:consent_group)&lt;-[:of_participant]-(:participant)&lt;-[:of_sample]-(:sample)&lt;--(cp)&lt;--(sm2:sample)
+WHERE cp:cell_line OR cp:pdx
+WITH s, num_of_participants, num_samples_1 + count(DISTINCT sm2.sample_id) AS num_of_samples
+OPTIONAL MATCH (s)&lt;-[*..6]-(dg:diagnosis)
+WITH s, num_of_participants, num_of_samples, dg.diagnosis AS diagnosis_name, count(dg.diagnosis) AS diagnosis_n
+ORDER BY diagnosis_n DESC, diagnosis_name ASC
 WITH s, num_of_participants, num_of_samples,
      [item IN collect(CASE WHEN diagnosis_name IS NULL THEN null ELSE diagnosis_name + ' (' + toString(diagnosis_n) + ')' END) WHERE item IS NOT NULL] AS diagnosis_all
 WITH s, num_of_participants, num_of_samples,
      diagnosis_all[0..5] AS diagnosis_items,
      size(diagnosis_all) &gt; 5 AS diagnosis_more
-OPTIONAL MATCH (d2:diagnosis)-[:of_diagnosis]-&gt;(dp2:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
-UNWIND CASE
-  WHEN d2 IS NULL THEN []
-  WHEN size(coalesce(d2.anatomic_site, [])) = 0 THEN [null]
-  ELSE d2.anatomic_site
-END AS site_raw
-WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, d2, site_raw,
+OPTIONAL MATCH (s)&lt;-[*..6]-(diag:diagnosis)
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more,
+     coalesce(diag.anatomic_site, []) AS dg_sites
+UNWIND CASE WHEN size(dg_sites) = 0 THEN [null] ELSE dg_sites END AS site_raw
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more,
      CASE
        WHEN site_raw IS NULL OR trim(toString(site_raw)) = '' THEN 'Not Reported'
        ELSE site_raw
      END AS site
-WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site, count(DISTINCT d2) AS site_n
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site, count(site) AS site_n
 ORDER BY site_n DESC, site ASC
 WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more,
      collect(site + ' (' + toString(site_n) + ')') AS site_all
@@ -591,13 +613,15 @@
 WHERE (fl:clinical_measure_file OR fl:generic_file OR fl:sequencing_file OR fl:pathology_file OR fl:radiology_file OR fl:methylation_array_file OR fl:cytogenomic_file)
 WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more,
      fl.file_type AS file_type, count(DISTINCT fl.dcf_indexd_guid) AS type_n
-ORDER BY type_n DESC
+ORDER BY type_n DESC, file_type ASC
 WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more,
      sum(CASE WHEN file_type IS NULL THEN 0 ELSE type_n END) AS num_of_files,
      [item IN collect(CASE WHEN file_type IS NULL THEN null ELSE file_type + ' (' + toString(type_n) + ')' END) WHERE item IS NOT NULL] AS file_type_all
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more, num_of_files, file_type_all,
+     [item IN file_type_all WHERE NOT item STARTS WITH 'crai ('] AS file_type_filtered
 WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more, num_of_files,
-     file_type_all[0..5] AS file_type_items,
-     size(file_type_all) &gt; 5 AS file_type_more
+     file_type_filtered[0..5] AS file_type_items,
+     size(file_type_filtered) &gt; 5 AS file_type_more
 OPTIONAL MATCH (pub:publication)-[:of_publication]-&gt;(s)
 WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more, num_of_files, file_type_items, file_type_more,
      [id IN collect(pub.pubmed_id) WHERE id IS NOT NULL] AS pubmed_ids
@@ -607,7 +631,7 @@
      [name IN collect(per.personnel_name) WHERE name IS NOT NULL] AS investigators
 OPTIONAL MATCH (fund:study_funding)-[:of_study_funding]-&gt;(s)
 WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site_items, site_more, num_of_files, file_type_items, file_type_more, pubmed_ids, investigators,
-     [id IN collect(fund.grant_id) WHERE id IS NOT NULL] AS grant_ids
+     [id IN collect(DISTINCT fund.grant_id) WHERE id IS NOT NULL] AS grant_ids
 RETURN s.study_name AS `Study Name`,
        s.study_id AS `Study ID`,
        s.study_phase AS `Study Phase`,
@@ -802,9 +826,24 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">MATCH (sm:sample)-[:of_sample]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
+          <t>CALL {
+  MATCH (sm:sample)-[:of_sample]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
+  WHERE s.dbgap_accession = 'phs002430' AND p.sex_at_birth = 'Unknown'
+  RETURN sm, p
+  UNION
+  MATCH (parent:sample)-[:of_sample]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
+  WHERE s.dbgap_accession = 'phs002430' AND p.sex_at_birth = 'Unknown'
+  MATCH (sm:sample)-[:of_sample]-&gt;(:cell_line)-[:of_cell_line]-&gt;(parent)
+  RETURN sm, p
+  UNION
+  MATCH (parent:sample)-[:of_sample]-&gt;(p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
+  WHERE s.dbgap_accession = 'phs002430' AND p.sex_at_birth = 'Unknown'
+  MATCH (sm:sample)-[:of_sample]-&gt;(:pdx)-[:of_pdx]-&gt;(parent)
+  RETURN sm, p
+}
+WITH DISTINCT sm, p
+MATCH (p)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
 WHERE s.dbgap_accession = 'phs002430'
-  AND p.sex_at_birth = 'Unknown'
 RETURN p.participant_id AS `Participant ID`,
        sm.sample_id AS `Sample ID`,
        s.study_id AS `Study ID`,
@@ -816,8 +855,7 @@
        END AS `Participant Age at Collection (days)`,
        sm.sample_tumor_status AS `Sample Tumor Status`
 ORDER BY sm.sample_id
-LIMIT 100;
-</t>
+LIMIT 100;</t>
         </is>
       </c>
     </row>

</xml_diff>